<commit_message>
Net partner debt payments against expense overpay clawback
Adds settlement math: his unpaid half of shop-paid bills minus proven
debt sends equals net still owed, separate from the $30k capital gap.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/cesar-money-clawback.xlsx
+++ b/finance/cesar-money-clawback.xlsx
@@ -53,7 +53,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +78,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1E7DD"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -131,6 +136,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -496,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -663,6 +670,22 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Debt payments he already sent you (proven)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Venmo/Zelle he called “debt payback” — evidence only</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -1018,12 +1041,149 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>NET SETTLEMENT (your idea — correct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="55" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>You overpaid his half of expenses from the shop account. Any money he already sent as “debt” gets subtracted from that overpay. Only the NET still owed is what he writes a check for on expenses. Capital to hit $30k stays a SEPARATE line (don’t mix unless you agree to apply debt payments to capital instead).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>You overpaid (his 50% of shop-paid bills)</t>
+        </is>
+      </c>
+      <c r="B53" s="9">
+        <f>B27</f>
+        <v/>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Clawback before credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Minus: debt payments he already sent (proven)</t>
+        </is>
+      </c>
+      <c r="B54" s="6">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Credit against clawback</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>NET expense clawback still owed to you</t>
+        </is>
+      </c>
+      <c r="B55" s="10">
+        <f>MAX(0,B27-B14)</f>
+        <v/>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Check he still owes for expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>If debt payments exceed clawback (leftover credit)</t>
+        </is>
+      </c>
+      <c r="B56" s="18">
+        <f>MAX(0,B14-B27)</f>
+        <v/>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Can apply to his $30k capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Capital still needed for $30k</t>
+        </is>
+      </c>
+      <c r="B57" s="9">
+        <f>MAX(0,B12-B13)</f>
+        <v/>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Separate line</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL still owed (net clawback + capital gap)</t>
+        </is>
+      </c>
+      <c r="B58" s="10">
+        <f>B55+B57</f>
+        <v/>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Sit-down number</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Example with defaults: overpay $7,500. If he already Venmo’d you $2,000 as “debt,” net clawback = $5,500. Then capital gap to $30k is still whatever documented capital is short.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="A49:C49"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A50:C50"/>
     <mergeCell ref="A47:D47"/>
     <mergeCell ref="A44:D44"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add \$1250 vs \$625 three-month shortfall calc to clawback sheet
Clarifies monthly net as half-of-bills minus his \$625 credit, times
three months, so Cesar can pick that framing without double-counting.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/cesar-money-clawback.xlsx
+++ b/finance/cesar-money-clawback.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -685,7 +685,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -1175,16 +1174,136 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>ALTERNATE (your 625 vs 1250 × 3 months)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="55" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>You said: he “gets” $625/mo, half of bills is $1,250/mo, for 3 months. Correct order is: he owes $1,250 − $625 = $625 per month (not 625−1250). × 3 months = $1,875 — UNLESS the $625 was actual cash he already paid in, in which case same math: credit $625 against his $1,250 half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>Input / result</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C65" s="17" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>His half of monthly burn (50% of $2,500)</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>What he should pay each month</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Credit / “he gets” each month</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="n">
+        <v>625</v>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>25% share credit OR cash he already put in — edit</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Months this applied</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>You said 3 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>Monthly shortfall he owes</t>
+        </is>
+      </c>
+      <c r="B69" s="9">
+        <f>B66-B67</f>
+        <v/>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>$1,250 − $625</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL from this 3-month rule</t>
+        </is>
+      </c>
+      <c r="B70" s="10">
+        <f>B69*B68</f>
+        <v/>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Sit-down number under THIS framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="70" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Which method to use?
+• Full clawback: 50% × ALL months bills were paid from shop account (6×$2,500 → $7,500), then subtract debt Venmos.
+• This 3-month net: only the months you agree the $625 credit applies → $1,875.
+Don’t double-count: if you use the $1,875 method, don’t also charge full $7,500 for those same 3 months.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A60:C60"/>
     <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A63:C63"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A50:C50"/>
     <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A72:C72"/>
     <mergeCell ref="A44:D44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add business-logic sheet for 20%-to-50% expense gap
Frames break-even, investor pocket pain, and Alexis's 30% funding gap
as accounting so Cesar's sit-down numbers stay calm and consistent.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/cesar-money-clawback.xlsx
+++ b/finance/cesar-money-clawback.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Clawback" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="MonthByMonth" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BusinessLogic" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Clawback" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthByMonth" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +53,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -85,6 +91,11 @@
         <fgColor rgb="00D1E7DD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -112,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -138,6 +149,10 @@
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -503,6 +518,331 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Why the numbers have to work this way (not a fight — accounting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>THE SITUATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>1) Shop is break-even → after rent/expenses there is $0 leftover.
+2) $0 leftover means $0 profit draw to send your investor from operations.
+3) If you still pay the investor, that cash is coming out of YOUR pocket — while your capital is already tied up in the chairs/shop.
+4) You and Alexis invested together, but he only put ~20% down.
+5) You are sitting the deal at $60k = $30k each (50/50). His 20% → 50% is a 30% GAP.
+6) That 30% of monthly bills has to come from HIS pocket. If it instead clears the business account funded by your money, you paid his gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Monthly burn (rent + expenses)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $1,700 + ~$800</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>His capital in (what he actually put down)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>He put ~20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Target equal share (new deal)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>$30k / $30k</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Gap he must fund (50% − 20%)</t>
+        </is>
+      </c>
+      <c r="B11" s="20">
+        <f>B10-B9</f>
+        <v/>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>The 30% gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Months bills paid from business account</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Use 3 or 6 — edit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Credit already given him per month (optional)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>625</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>If you credited him $625/mo; else set 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>CLEAN MATH</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>His gap $ per month (30% × burn)</t>
+        </is>
+      </c>
+      <c r="B17" s="12">
+        <f>B8*B11</f>
+        <v/>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>What must come from HIS pocket each month</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>His full 50% half of burn</t>
+        </is>
+      </c>
+      <c r="B18" s="9">
+        <f>B8*B10</f>
+        <v/>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>$1,250 if burn is $2,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>His 20% share of burn only</t>
+        </is>
+      </c>
+      <c r="B19" s="9">
+        <f>B8*B9</f>
+        <v/>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>$500 if burn is $2,500 — ownership matching 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>If you already credited him $625/mo, extra shortfall</t>
+        </is>
+      </c>
+      <c r="B20" s="9">
+        <f>MAX(0,B18-B13)</f>
+        <v/>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>$1,250 − $625</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL gap owed (30% × burn × months)</t>
+        </is>
+      </c>
+      <c r="B21" s="21">
+        <f>B17*B12</f>
+        <v/>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Business true-up for the gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL using 50% − $625 credit × months</t>
+        </is>
+      </c>
+      <c r="B22" s="21">
+        <f>B20*B12</f>
+        <v/>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Your 3-month net framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>HOW THIS TIES TO THE INVESTOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="85" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Chairs/shop = the investment asset. No monthly profit = operations cannot fund investor returns.
+Paying the investor from your pocket while also covering Alexis’s unpaid 30% gap means you are funding BOTH the investor AND his missing capital/expense share.
+Fix (business, not personal): he funds the 30% gap from his pocket (or buys up to 50% / $30k documented). Shop account stops covering his gap. Then your pocket is only dealing with investor + your own 50%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>One-sentence version for the sit-down</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>"We're at $60k / $30k each. You put in ~20%, so until you're at 50% documented, the 30% gap on bills comes from your pocket — not the shop account — because the account is my capital and there's no profit left after rent. I'm not fighting you; the books have to match the deal."</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>With defaults ($2,500 burn, 30% gap, 3 months): gap = $750/mo × 3 = $2,250. With $625 credit framing: $625/mo × 3 = $1,875.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A28:D28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1310,7 +1650,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>